<commit_message>
Fix covenant forecast task
</commit_message>
<xml_diff>
--- a/companies/alder-ridge/source-files/Shared/Finance/Treasury/Bank - covenants/FY27 covenant forecast - WORKING.xlsx
+++ b/companies/alder-ridge/source-files/Shared/Finance/Treasury/Bank - covenants/FY27 covenant forecast - WORKING.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast Inputs" sheetId="1" r:id="R0a64ebf6b5c14cb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule" sheetId="2" r:id="Rbe70ad39e6d24f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenant Forecast" sheetId="3" r:id="R177ece3ac858440d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downside" sheetId="4" r:id="Re40d85d4025b422c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="R5ea44deb7d2c403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast Inputs" sheetId="1" r:id="Rb419116265204649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule" sheetId="2" r:id="R4babc73c4be249e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covenant Forecast" sheetId="3" r:id="R9ff1fcc6bc114be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downside" sheetId="4" r:id="R9cef0839a2d34a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="R845b00f7c64142a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,7 +256,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Alder Ridge Finance" id="{9ACB837F-539F-4ABA-AF7F-4432F0A5EF44}"/>
+  <xltc:person displayName="Alder Ridge Finance" id="{985C9149-0327-48D7-8FF3-3DEAF244E7DB}"/>
 </xltc:personList>
 </file>
 
@@ -624,7 +624,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G7" s="26" t="n">
         <x:v>620000</x:v>
@@ -828,7 +828,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F13" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G13" s="26" t="n">
         <x:v>620000</x:v>
@@ -1032,7 +1032,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G19" s="26" t="n">
         <x:v>620000</x:v>
@@ -1236,7 +1236,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F25" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G25" s="26" t="n">
         <x:v>870000</x:v>
@@ -1440,7 +1440,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G31" s="26" t="n">
         <x:v>620000</x:v>
@@ -1644,7 +1644,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G37" s="26" t="n">
         <x:v>620000</x:v>
@@ -1848,7 +1848,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G43" s="26" t="n">
         <x:v>620000</x:v>
@@ -2052,7 +2052,7 @@
         <x:v>Approved case</x:v>
       </x:c>
       <x:c r="F49" s="23" t="str">
-        <x:v>Capital expenditures</x:v>
+        <x:v>Unfunded capital expenditures</x:v>
       </x:c>
       <x:c r="G49" s="26" t="n">
         <x:v>870000</x:v>
@@ -2240,38 +2240,548 @@
       <x:c r="L54" s="23" t="str"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="24" t="str">
+      <x:c r="A55" s="23" t="str">
         <x:v>048-SRC0053</x:v>
       </x:c>
-      <x:c r="B55" s="24" t="str">
+      <x:c r="B55" s="23" t="str">
         <x:v>Covenant policy</x:v>
       </x:c>
-      <x:c r="C55" s="24" t="str">
+      <x:c r="C55" s="23" t="str">
         <x:v>Credit agreement</x:v>
       </x:c>
-      <x:c r="D55" s="24" t="str">
+      <x:c r="D55" s="23" t="str">
         <x:v>Forecast horizon</x:v>
       </x:c>
-      <x:c r="E55" s="24" t="str">
-        <x:v>Approved case</x:v>
-      </x:c>
-      <x:c r="F55" s="24" t="str">
+      <x:c r="E55" s="23" t="str">
+        <x:v>Approved case</x:v>
+      </x:c>
+      <x:c r="F55" s="23" t="str">
         <x:v>Minimum quarterly capex deduction</x:v>
       </x:c>
-      <x:c r="G55" s="27" t="n">
+      <x:c r="G55" s="26" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H55" s="24" t="str"/>
-      <x:c r="I55" s="24" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="J55" s="24" t="str">
-        <x:v>Finance operating schedule</x:v>
-      </x:c>
-      <x:c r="K55" s="30" t="str">
-        <x:v>2026-06-30</x:v>
-      </x:c>
-      <x:c r="L55" s="24" t="str"/>
+      <x:c r="H55" s="23" t="str"/>
+      <x:c r="I55" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J55" s="23" t="str">
+        <x:v>Finance operating schedule</x:v>
+      </x:c>
+      <x:c r="K55" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L55" s="23" t="str"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="23" t="str">
+        <x:v>048-SRC0054</x:v>
+      </x:c>
+      <x:c r="B56" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C56" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D56" s="23" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="E56" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F56" s="23" t="str">
+        <x:v>Quarterly covenant EBITDA</x:v>
+      </x:c>
+      <x:c r="G56" s="26" t="n">
+        <x:v>2850000</x:v>
+      </x:c>
+      <x:c r="H56" s="23" t="str"/>
+      <x:c r="I56" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J56" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K56" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L56" s="23" t="str"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="23" t="str">
+        <x:v>048-SRC0055</x:v>
+      </x:c>
+      <x:c r="B57" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C57" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D57" s="23" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="E57" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F57" s="23" t="str">
+        <x:v>Cash interest</x:v>
+      </x:c>
+      <x:c r="G57" s="26" t="n">
+        <x:v>416000</x:v>
+      </x:c>
+      <x:c r="H57" s="23" t="str"/>
+      <x:c r="I57" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J57" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K57" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L57" s="23" t="str"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="23" t="str">
+        <x:v>048-SRC0056</x:v>
+      </x:c>
+      <x:c r="B58" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C58" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D58" s="23" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="E58" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F58" s="23" t="str">
+        <x:v>Unfunded capital expenditures</x:v>
+      </x:c>
+      <x:c r="G58" s="26" t="n">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="H58" s="23" t="str"/>
+      <x:c r="I58" s="23" t="str">
+        <x:v>USD thousands</x:v>
+      </x:c>
+      <x:c r="J58" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K58" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L58" s="23" t="str"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="23" t="str">
+        <x:v>048-SRC0057</x:v>
+      </x:c>
+      <x:c r="B59" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C59" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D59" s="23" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="E59" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F59" s="23" t="str">
+        <x:v>Cash taxes</x:v>
+      </x:c>
+      <x:c r="G59" s="26" t="n">
+        <x:v>280000</x:v>
+      </x:c>
+      <x:c r="H59" s="23" t="str"/>
+      <x:c r="I59" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J59" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K59" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L59" s="23" t="str"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="23" t="str">
+        <x:v>048-SRC0058</x:v>
+      </x:c>
+      <x:c r="B60" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C60" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D60" s="23" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="E60" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F60" s="23" t="str">
+        <x:v>Scheduled debt repayment</x:v>
+      </x:c>
+      <x:c r="G60" s="26" t="n">
+        <x:v>650000</x:v>
+      </x:c>
+      <x:c r="H60" s="23" t="str"/>
+      <x:c r="I60" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J60" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K60" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L60" s="23" t="str"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="23" t="str">
+        <x:v>048-SRC0059</x:v>
+      </x:c>
+      <x:c r="B61" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C61" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D61" s="23" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="E61" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F61" s="23" t="str">
+        <x:v>Quarterly covenant EBITDA</x:v>
+      </x:c>
+      <x:c r="G61" s="26" t="n">
+        <x:v>2920000</x:v>
+      </x:c>
+      <x:c r="H61" s="23" t="str"/>
+      <x:c r="I61" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J61" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K61" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L61" s="23" t="str"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="23" t="str">
+        <x:v>048-SRC0060</x:v>
+      </x:c>
+      <x:c r="B62" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C62" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D62" s="23" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="E62" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F62" s="23" t="str">
+        <x:v>Cash interest</x:v>
+      </x:c>
+      <x:c r="G62" s="26" t="n">
+        <x:v>434</x:v>
+      </x:c>
+      <x:c r="H62" s="23" t="str"/>
+      <x:c r="I62" s="23" t="str">
+        <x:v>USD thousands</x:v>
+      </x:c>
+      <x:c r="J62" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K62" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L62" s="23" t="str"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="23" t="str">
+        <x:v>048-SRC0061</x:v>
+      </x:c>
+      <x:c r="B63" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C63" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D63" s="23" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="E63" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F63" s="23" t="str">
+        <x:v>Unfunded capital expenditures</x:v>
+      </x:c>
+      <x:c r="G63" s="26" t="n">
+        <x:v>610000</x:v>
+      </x:c>
+      <x:c r="H63" s="23" t="str"/>
+      <x:c r="I63" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J63" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K63" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L63" s="23" t="str"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="23" t="str">
+        <x:v>048-SRC0062</x:v>
+      </x:c>
+      <x:c r="B64" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C64" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D64" s="23" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="E64" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F64" s="23" t="str">
+        <x:v>Cash taxes</x:v>
+      </x:c>
+      <x:c r="G64" s="26" t="n">
+        <x:v>290000</x:v>
+      </x:c>
+      <x:c r="H64" s="23" t="str"/>
+      <x:c r="I64" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J64" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K64" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L64" s="23" t="str"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="23" t="str">
+        <x:v>048-SRC0063</x:v>
+      </x:c>
+      <x:c r="B65" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C65" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D65" s="23" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="E65" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F65" s="23" t="str">
+        <x:v>Scheduled debt repayment</x:v>
+      </x:c>
+      <x:c r="G65" s="26" t="n">
+        <x:v>650000</x:v>
+      </x:c>
+      <x:c r="H65" s="23" t="str"/>
+      <x:c r="I65" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J65" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K65" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L65" s="23" t="str"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="23" t="str">
+        <x:v>048-SRC0064</x:v>
+      </x:c>
+      <x:c r="B66" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C66" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D66" s="23" t="str">
+        <x:v>2026-Q2</x:v>
+      </x:c>
+      <x:c r="E66" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F66" s="23" t="str">
+        <x:v>Quarterly covenant EBITDA</x:v>
+      </x:c>
+      <x:c r="G66" s="26" t="n">
+        <x:v>3010</x:v>
+      </x:c>
+      <x:c r="H66" s="23" t="str"/>
+      <x:c r="I66" s="23" t="str">
+        <x:v>USD thousands</x:v>
+      </x:c>
+      <x:c r="J66" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K66" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L66" s="23" t="str"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="23" t="str">
+        <x:v>048-SRC0065</x:v>
+      </x:c>
+      <x:c r="B67" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C67" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D67" s="23" t="str">
+        <x:v>2026-Q2</x:v>
+      </x:c>
+      <x:c r="E67" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F67" s="23" t="str">
+        <x:v>Cash interest</x:v>
+      </x:c>
+      <x:c r="G67" s="26" t="n">
+        <x:v>452000</x:v>
+      </x:c>
+      <x:c r="H67" s="23" t="str"/>
+      <x:c r="I67" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J67" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K67" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L67" s="23" t="str"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="23" t="str">
+        <x:v>048-SRC0066</x:v>
+      </x:c>
+      <x:c r="B68" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C68" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D68" s="23" t="str">
+        <x:v>2026-Q2</x:v>
+      </x:c>
+      <x:c r="E68" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F68" s="23" t="str">
+        <x:v>Unfunded capital expenditures</x:v>
+      </x:c>
+      <x:c r="G68" s="26" t="n">
+        <x:v>620000</x:v>
+      </x:c>
+      <x:c r="H68" s="23" t="str"/>
+      <x:c r="I68" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J68" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K68" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L68" s="23" t="str"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="23" t="str">
+        <x:v>048-SRC0067</x:v>
+      </x:c>
+      <x:c r="B69" s="23" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C69" s="23" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D69" s="23" t="str">
+        <x:v>2026-Q2</x:v>
+      </x:c>
+      <x:c r="E69" s="23" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F69" s="23" t="str">
+        <x:v>Cash taxes</x:v>
+      </x:c>
+      <x:c r="G69" s="26" t="n">
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="H69" s="23" t="str"/>
+      <x:c r="I69" s="23" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J69" s="23" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K69" s="29" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L69" s="23" t="str"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="24" t="str">
+        <x:v>048-SRC0068</x:v>
+      </x:c>
+      <x:c r="B70" s="24" t="str">
+        <x:v>Historical Covenant Inputs</x:v>
+      </x:c>
+      <x:c r="C70" s="24" t="str">
+        <x:v>Consolidated</x:v>
+      </x:c>
+      <x:c r="D70" s="24" t="str">
+        <x:v>2026-Q2</x:v>
+      </x:c>
+      <x:c r="E70" s="24" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="F70" s="24" t="str">
+        <x:v>Scheduled debt repayment</x:v>
+      </x:c>
+      <x:c r="G70" s="27" t="n">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="H70" s="24" t="str"/>
+      <x:c r="I70" s="24" t="str">
+        <x:v>USD thousands</x:v>
+      </x:c>
+      <x:c r="J70" s="24" t="str">
+        <x:v>Q2 covenant history - controller tie</x:v>
+      </x:c>
+      <x:c r="K70" s="30" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+      <x:c r="L70" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>